<commit_message>
Experiments without CacheSaver works
</commit_message>
<xml_diff>
--- a/math/experiment_results.xlsx
+++ b/math/experiment_results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/89c2773904d5ab9b/Dokumenter/Datalogi/Semester 6/Bachelor/llm_multiagent_debate_cachesaver-1/math/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="11_2B59D2BFD340DA84E85FA7104F3088B35299F083" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7363A34E-4485-43F1-B8A4-818BDFAE535A}"/>
+  <xr:revisionPtr revIDLastSave="26" documentId="11_2B59D2BFD3F0DDCEF2E15C134C3088B35299F08B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AE12B296-3494-48F9-9486-62CAEBEB82E8}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>agents</t>
   </si>
@@ -46,7 +46,16 @@
     <t>total_tokens</t>
   </si>
   <si>
-    <t>runtime</t>
+    <t>runtime (s)</t>
+  </si>
+  <si>
+    <t>Model</t>
+  </si>
+  <si>
+    <t>qwen2.5:1.5b</t>
+  </si>
+  <si>
+    <t>qwen3:0.6b</t>
   </si>
 </sst>
 </file>
@@ -75,7 +84,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -98,13 +107,27 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -409,18 +432,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="20.44140625" customWidth="1"/>
-    <col min="5" max="5" width="11.109375" customWidth="1"/>
-    <col min="6" max="6" width="18" customWidth="1"/>
-    <col min="7" max="7" width="17.109375" customWidth="1"/>
-    <col min="8" max="8" width="16.88671875" customWidth="1"/>
+    <col min="1" max="1" width="8.88671875" customWidth="1"/>
+    <col min="2" max="2" width="9" customWidth="1"/>
+    <col min="3" max="3" width="18.6640625" customWidth="1"/>
+    <col min="4" max="4" width="18.77734375" customWidth="1"/>
+    <col min="5" max="5" width="16.21875" customWidth="1"/>
+    <col min="6" max="6" width="17.44140625" customWidth="1"/>
+    <col min="7" max="7" width="17.5546875" customWidth="1"/>
+    <col min="8" max="8" width="20" customWidth="1"/>
+    <col min="9" max="9" width="15.44140625" customWidth="1"/>
+    <col min="10" max="10" width="17.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -448,8 +475,11 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
+      <c r="J1" s="2" t="s">
+        <v>9</v>
+      </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -469,16 +499,19 @@
         <v>45</v>
       </c>
       <c r="G2">
-        <v>1182</v>
+        <v>785</v>
       </c>
       <c r="H2">
-        <v>1227</v>
+        <v>830</v>
       </c>
       <c r="I2">
-        <v>8</v>
+        <v>5.82</v>
+      </c>
+      <c r="J2" t="s">
+        <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -495,19 +528,19 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>731</v>
+        <v>474</v>
       </c>
       <c r="G3">
-        <v>756</v>
+        <v>855</v>
       </c>
       <c r="H3">
-        <v>1487</v>
+        <v>1329</v>
       </c>
       <c r="I3">
-        <v>34</v>
+        <v>21.95</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -521,19 +554,109 @@
         <v>0</v>
       </c>
       <c r="E4">
-        <v>0.67</v>
+        <v>0</v>
       </c>
       <c r="F4">
-        <v>3992</v>
+        <v>2613</v>
       </c>
       <c r="G4">
-        <v>1176</v>
+        <v>1388</v>
       </c>
       <c r="H4">
-        <v>5168</v>
+        <v>4001</v>
       </c>
       <c r="I4">
-        <v>76</v>
+        <v>76.66</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>1</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6" t="b">
+        <v>0</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6">
+        <v>64</v>
+      </c>
+      <c r="G6">
+        <v>224</v>
+      </c>
+      <c r="H6">
+        <v>288</v>
+      </c>
+      <c r="I6">
+        <v>6.25</v>
+      </c>
+      <c r="J6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>2</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7">
+        <v>2</v>
+      </c>
+      <c r="D7" t="b">
+        <v>0</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="F7">
+        <v>1774</v>
+      </c>
+      <c r="G7">
+        <v>419</v>
+      </c>
+      <c r="H7">
+        <v>2193</v>
+      </c>
+      <c r="I7">
+        <v>14.19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>3</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8">
+        <v>3</v>
+      </c>
+      <c r="D8" t="b">
+        <v>0</v>
+      </c>
+      <c r="E8">
+        <v>0.33</v>
+      </c>
+      <c r="F8">
+        <v>11587</v>
+      </c>
+      <c r="G8">
+        <v>377</v>
+      </c>
+      <c r="H8">
+        <v>11964</v>
+      </c>
+      <c r="I8">
+        <v>36.93</v>
       </c>
     </row>
   </sheetData>

</xml_diff>